<commit_message>
Lotsofassembly-comments Added extra MCS48-info Updated Excelsheet
</commit_message>
<xml_diff>
--- a/Data/PM2528 Technical details.xlsx
+++ b/Data/PM2528 Technical details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF263DB-48F4-437C-8D7F-AE003239EF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B668C8F4-C42D-4347-9A42-9203E1C22721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
   <sheets>
     <sheet name="MainBoard-Relais" sheetId="3" r:id="rId1"/>
@@ -722,15 +722,9 @@
     <t>0xf0</t>
   </si>
   <si>
-    <t>something with Galvanic Isolation Card</t>
-  </si>
-  <si>
     <t>1 = N30.R3019=1, Galvanic type 1</t>
   </si>
   <si>
-    <t>Statemachine?</t>
-  </si>
-  <si>
     <t>A3</t>
   </si>
   <si>
@@ -779,18 +773,9 @@
     <t>Autoranging</t>
   </si>
   <si>
-    <t>Bitpattern for Function-indicators</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>0000=VDC, 0001=VAC, 0010=VDCAC, 0011=O2W</t>
-  </si>
-  <si>
-    <t>00100=O4W, 00101ADC, 0110=ADCAC, 0111=C</t>
-  </si>
-  <si>
     <t>1000=Vhf, 1001=Vpeak</t>
   </si>
   <si>
@@ -825,6 +810,21 @@
   </si>
   <si>
     <t>`</t>
+  </si>
+  <si>
+    <t>Datahold active?</t>
+  </si>
+  <si>
+    <t>Currently selected function-indx</t>
+  </si>
+  <si>
+    <t>??1010=Vhf-without-module, 1011=Vpeak-without-module</t>
+  </si>
+  <si>
+    <t>0000=VDC, 0001=VAC, 0010=VDCAC, 0011=R2W</t>
+  </si>
+  <si>
+    <t>00100=R4W, 00101ADC, 0110=ADCAC, 0111=C</t>
   </si>
 </sst>
 </file>
@@ -920,12 +920,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -945,6 +939,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1281,22 +1281,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -1308,42 +1307,43 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1710,78 +1710,78 @@
       <c r="BE1" s="3"/>
     </row>
     <row r="2" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="C2" s="61" t="s">
+      <c r="C2" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="61" t="s">
+      <c r="I2" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="M2" s="61"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="60"/>
       <c r="N2" s="3"/>
-      <c r="O2" s="61" t="s">
+      <c r="O2" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="P2" s="61"/>
-      <c r="Q2" s="61"/>
-      <c r="R2" s="61"/>
-      <c r="S2" s="61"/>
+      <c r="P2" s="60"/>
+      <c r="Q2" s="60"/>
+      <c r="R2" s="60"/>
+      <c r="S2" s="60"/>
       <c r="T2" s="3"/>
-      <c r="U2" s="61" t="s">
+      <c r="U2" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="V2" s="61"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="61"/>
-      <c r="Y2" s="61"/>
-      <c r="Z2" s="61"/>
-      <c r="AA2" s="61"/>
-      <c r="AB2" s="61"/>
+      <c r="V2" s="60"/>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
+      <c r="Y2" s="60"/>
+      <c r="Z2" s="60"/>
+      <c r="AA2" s="60"/>
+      <c r="AB2" s="60"/>
       <c r="AC2" s="3"/>
-      <c r="AD2" s="61" t="s">
+      <c r="AD2" s="60" t="s">
         <v>34</v>
       </c>
-      <c r="AE2" s="61"/>
-      <c r="AF2" s="61"/>
-      <c r="AG2" s="61"/>
-      <c r="AH2" s="61"/>
+      <c r="AE2" s="60"/>
+      <c r="AF2" s="60"/>
+      <c r="AG2" s="60"/>
+      <c r="AH2" s="60"/>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="61" t="s">
+      <c r="AJ2" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="AK2" s="61"/>
-      <c r="AL2" s="61"/>
-      <c r="AM2" s="61"/>
-      <c r="AN2" s="61"/>
-      <c r="AO2" s="61"/>
-      <c r="AP2" s="61"/>
+      <c r="AK2" s="60"/>
+      <c r="AL2" s="60"/>
+      <c r="AM2" s="60"/>
+      <c r="AN2" s="60"/>
+      <c r="AO2" s="60"/>
+      <c r="AP2" s="60"/>
       <c r="AQ2" s="3"/>
-      <c r="AR2" s="61" t="s">
+      <c r="AR2" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="AS2" s="61"/>
-      <c r="AT2" s="61"/>
-      <c r="AU2" s="61"/>
-      <c r="AV2" s="61"/>
-      <c r="AW2" s="61"/>
-      <c r="AX2" s="61"/>
+      <c r="AS2" s="60"/>
+      <c r="AT2" s="60"/>
+      <c r="AU2" s="60"/>
+      <c r="AV2" s="60"/>
+      <c r="AW2" s="60"/>
+      <c r="AX2" s="60"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="BA2" s="3"/>
-      <c r="BB2" s="61" t="s">
+      <c r="BB2" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="BC2" s="61"/>
-      <c r="BD2" s="61"/>
+      <c r="BC2" s="60"/>
+      <c r="BD2" s="60"/>
       <c r="BE2" s="3"/>
       <c r="BF2" s="41" t="s">
         <v>43</v>
@@ -7000,69 +7000,69 @@
       </c>
     </row>
     <row r="2" spans="1:29" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D2" s="64" t="s">
+      <c r="D2" s="63" t="s">
         <v>134</v>
       </c>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
-      <c r="P2" s="64"/>
-      <c r="Q2" s="64"/>
-      <c r="R2" s="64"/>
-      <c r="S2" s="64"/>
-      <c r="T2" s="64"/>
-      <c r="U2" s="64"/>
-      <c r="V2" s="64"/>
-      <c r="W2" s="64"/>
-      <c r="X2" s="64"/>
-      <c r="Y2" s="64"/>
-      <c r="Z2" s="64"/>
-      <c r="AA2" s="64"/>
-      <c r="AB2" s="64"/>
-      <c r="AC2" s="64"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="63"/>
+      <c r="N2" s="63"/>
+      <c r="O2" s="63"/>
+      <c r="P2" s="63"/>
+      <c r="Q2" s="63"/>
+      <c r="R2" s="63"/>
+      <c r="S2" s="63"/>
+      <c r="T2" s="63"/>
+      <c r="U2" s="63"/>
+      <c r="V2" s="63"/>
+      <c r="W2" s="63"/>
+      <c r="X2" s="63"/>
+      <c r="Y2" s="63"/>
+      <c r="Z2" s="63"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="D3" s="65" t="s">
+      <c r="D3" s="64" t="s">
         <v>135</v>
       </c>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="63"/>
-      <c r="N3" s="66" t="s">
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="62"/>
+      <c r="N3" s="65" t="s">
         <v>113</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="66"/>
       <c r="R3" s="18"/>
-      <c r="S3" s="67" t="s">
+      <c r="S3" s="66" t="s">
         <v>114</v>
       </c>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="68"/>
-      <c r="X3" s="65" t="s">
+      <c r="T3" s="66"/>
+      <c r="U3" s="66"/>
+      <c r="V3" s="67"/>
+      <c r="X3" s="64" t="s">
         <v>49</v>
       </c>
-      <c r="Y3" s="62"/>
-      <c r="Z3" s="62"/>
+      <c r="Y3" s="61"/>
+      <c r="Z3" s="61"/>
       <c r="AA3" s="17"/>
-      <c r="AB3" s="62" t="s">
+      <c r="AB3" s="61" t="s">
         <v>50</v>
       </c>
-      <c r="AC3" s="63"/>
+      <c r="AC3" s="62"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="D4" s="22" t="s">
@@ -8531,7 +8531,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CF7209-D1EE-411E-A7B2-8C676C749DBA}">
-  <dimension ref="B1:AR36"/>
+  <dimension ref="B1:AQ36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -8539,72 +8539,70 @@
     <col min="10" max="10" width="2.5703125" customWidth="1"/>
     <col min="13" max="13" width="2.7109375" customWidth="1"/>
     <col min="14" max="14" width="10.5703125" customWidth="1"/>
-    <col min="19" max="19" width="9.140625" customWidth="1"/>
-    <col min="20" max="20" width="2.5703125" customWidth="1"/>
-    <col min="21" max="21" width="1.42578125" customWidth="1"/>
-    <col min="23" max="23" width="2.85546875" customWidth="1"/>
-    <col min="24" max="27" width="5.42578125" customWidth="1"/>
-    <col min="28" max="28" width="2.5703125" customWidth="1"/>
-    <col min="29" max="32" width="5.85546875" customWidth="1"/>
-    <col min="33" max="33" width="2.140625" customWidth="1"/>
-    <col min="34" max="37" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="2.7109375" customWidth="1"/>
-    <col min="40" max="43" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.28515625" customWidth="1"/>
+    <col min="20" max="20" width="1.42578125" customWidth="1"/>
+    <col min="22" max="22" width="2.85546875" customWidth="1"/>
+    <col min="23" max="26" width="5.42578125" customWidth="1"/>
+    <col min="27" max="27" width="2.5703125" customWidth="1"/>
+    <col min="28" max="31" width="5.85546875" customWidth="1"/>
+    <col min="32" max="32" width="2.140625" customWidth="1"/>
+    <col min="33" max="36" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="2.7109375" customWidth="1"/>
+    <col min="39" max="42" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:43" x14ac:dyDescent="0.25">
       <c r="S1" s="32"/>
-      <c r="U1" s="32"/>
-    </row>
-    <row r="2" spans="2:44" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="B2" s="64" t="s">
+      <c r="T1" s="32"/>
+    </row>
+    <row r="2" spans="2:43" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="B2" s="63" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
-      <c r="P2" s="64"/>
-      <c r="Q2" s="64"/>
-      <c r="R2" s="64"/>
-      <c r="S2" s="64"/>
-      <c r="T2" s="64"/>
-      <c r="U2" s="64"/>
-      <c r="V2" s="64"/>
-      <c r="W2" s="64"/>
-      <c r="X2" s="64"/>
-      <c r="Y2" s="64"/>
-      <c r="Z2" s="64"/>
-      <c r="AA2" s="64"/>
-      <c r="AB2" s="64"/>
-      <c r="AC2" s="64"/>
-      <c r="AD2" s="64"/>
-      <c r="AE2" s="64"/>
-      <c r="AF2" s="64"/>
-      <c r="AG2" s="64"/>
-      <c r="AH2" s="64"/>
-      <c r="AI2" s="64"/>
-      <c r="AJ2" s="64"/>
-      <c r="AK2" s="64"/>
-      <c r="AL2" s="64"/>
-      <c r="AM2" s="64"/>
-      <c r="AN2" s="64"/>
-      <c r="AO2" s="64"/>
-      <c r="AP2" s="64"/>
-      <c r="AQ2" s="64"/>
-      <c r="AR2" s="64"/>
-    </row>
-    <row r="3" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="63"/>
+      <c r="N2" s="63"/>
+      <c r="O2" s="63"/>
+      <c r="P2" s="63"/>
+      <c r="Q2" s="63"/>
+      <c r="R2" s="63"/>
+      <c r="S2" s="63"/>
+      <c r="T2" s="63"/>
+      <c r="U2" s="63"/>
+      <c r="V2" s="63"/>
+      <c r="W2" s="63"/>
+      <c r="X2" s="63"/>
+      <c r="Y2" s="63"/>
+      <c r="Z2" s="63"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
+      <c r="AD2" s="63"/>
+      <c r="AE2" s="63"/>
+      <c r="AF2" s="63"/>
+      <c r="AG2" s="63"/>
+      <c r="AH2" s="63"/>
+      <c r="AI2" s="63"/>
+      <c r="AJ2" s="63"/>
+      <c r="AK2" s="63"/>
+      <c r="AL2" s="63"/>
+      <c r="AM2" s="63"/>
+      <c r="AN2" s="63"/>
+      <c r="AO2" s="63"/>
+      <c r="AP2" s="63"/>
+      <c r="AQ2" s="63"/>
+    </row>
+    <row r="3" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B3" s="69" t="s">
         <v>204</v>
       </c>
@@ -8629,7 +8627,7 @@
       <c r="R3" s="69"/>
       <c r="S3" s="69"/>
     </row>
-    <row r="4" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
         <v>62</v>
       </c>
@@ -8680,7 +8678,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N5" t="s">
         <v>143</v>
       </c>
@@ -8699,9 +8697,9 @@
       <c r="S5" t="s">
         <v>142</v>
       </c>
-      <c r="U5" s="32"/>
-    </row>
-    <row r="6" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="T5" s="32"/>
+    </row>
+    <row r="6" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B6" s="32" t="s">
         <v>63</v>
       </c>
@@ -8750,9 +8748,9 @@
       <c r="S6" s="32">
         <v>1</v>
       </c>
-      <c r="U6" s="32"/>
-    </row>
-    <row r="7" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="T6" s="32"/>
+    </row>
+    <row r="7" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B7" s="32" t="s">
         <v>63</v>
       </c>
@@ -8778,7 +8776,7 @@
         <v>63</v>
       </c>
       <c r="K7" s="32" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="L7" s="32">
         <v>1</v>
@@ -8802,7 +8800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B8" s="32" t="s">
         <v>63</v>
       </c>
@@ -8852,7 +8850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B9" s="32" t="s">
         <v>63</v>
       </c>
@@ -8902,7 +8900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B10" s="32">
         <v>1</v>
       </c>
@@ -8933,10 +8931,10 @@
       <c r="L10" s="32">
         <v>1</v>
       </c>
-      <c r="N10" s="56">
-        <v>0</v>
-      </c>
-      <c r="O10" s="56">
+      <c r="N10" s="55">
+        <v>0</v>
+      </c>
+      <c r="O10" s="55">
         <v>0</v>
       </c>
       <c r="P10" s="32">
@@ -8952,7 +8950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B11" s="32">
         <v>1</v>
       </c>
@@ -8989,10 +8987,10 @@
       <c r="O11" s="32">
         <v>1</v>
       </c>
-      <c r="P11" s="56">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="56">
+      <c r="P11" s="55">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="55">
         <v>0</v>
       </c>
       <c r="R11" s="32">
@@ -9002,7 +9000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B12" s="32">
         <v>1</v>
       </c>
@@ -9045,14 +9043,14 @@
       <c r="Q12" s="32">
         <v>1</v>
       </c>
-      <c r="R12" s="56">
+      <c r="R12" s="55">
         <v>0</v>
       </c>
       <c r="S12" s="32">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:44" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B13" s="32">
         <v>1</v>
       </c>
@@ -9098,29 +9096,29 @@
       <c r="R13" s="32">
         <v>1</v>
       </c>
-      <c r="S13" s="56">
-        <v>0</v>
-      </c>
-      <c r="X13" s="70" t="s">
+      <c r="S13" s="55">
+        <v>0</v>
+      </c>
+      <c r="W13" s="72" t="s">
         <v>180</v>
       </c>
-      <c r="Y13" s="70"/>
-      <c r="Z13" s="70"/>
-    </row>
-    <row r="14" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="X13" s="72"/>
+      <c r="Y13" s="72"/>
+    </row>
+    <row r="14" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
       <c r="O14" s="32"/>
       <c r="P14" s="32"/>
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="X14" s="71" t="s">
+      <c r="W14" s="70" t="s">
         <v>197</v>
       </c>
-      <c r="Y14" s="71"/>
-      <c r="Z14" s="71"/>
-    </row>
-    <row r="15" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="X14" s="70"/>
+      <c r="Y14" s="70"/>
+    </row>
+    <row r="15" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
         <v>205</v>
       </c>
@@ -9129,13 +9127,13 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="X15" s="72" t="s">
+      <c r="W15" s="71" t="s">
         <v>198</v>
       </c>
-      <c r="Y15" s="72"/>
-      <c r="Z15" s="72"/>
-    </row>
-    <row r="16" spans="2:44" x14ac:dyDescent="0.25">
+      <c r="X15" s="71"/>
+      <c r="Y15" s="71"/>
+    </row>
+    <row r="16" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
       <c r="O16" s="32"/>
       <c r="P16" s="32"/>
@@ -9143,7 +9141,7 @@
       <c r="R16" s="32"/>
       <c r="S16" s="32"/>
     </row>
-    <row r="18" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="18" spans="14:43" x14ac:dyDescent="0.25">
       <c r="O18" s="69" t="s">
         <v>131</v>
       </c>
@@ -9153,10 +9151,10 @@
       <c r="S18" s="69"/>
       <c r="T18" s="69"/>
       <c r="U18" s="69"/>
-      <c r="V18" s="69"/>
-      <c r="X18" s="69" t="s">
+      <c r="W18" s="69" t="s">
         <v>181</v>
       </c>
+      <c r="X18" s="69"/>
       <c r="Y18" s="69"/>
       <c r="Z18" s="69"/>
       <c r="AA18" s="69"/>
@@ -9176,9 +9174,8 @@
       <c r="AO18" s="69"/>
       <c r="AP18" s="69"/>
       <c r="AQ18" s="69"/>
-      <c r="AR18" s="69"/>
-    </row>
-    <row r="19" spans="14:44" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="14:43" x14ac:dyDescent="0.25">
       <c r="O19" s="46" t="s">
         <v>171</v>
       </c>
@@ -9194,103 +9191,104 @@
       <c r="S19" s="46" t="s">
         <v>150</v>
       </c>
-      <c r="T19" s="46"/>
-      <c r="U19" s="57"/>
-      <c r="V19" s="46" t="s">
+      <c r="T19" s="56"/>
+      <c r="U19" s="46" t="s">
         <v>179</v>
       </c>
+      <c r="W19" s="46" t="s">
+        <v>151</v>
+      </c>
       <c r="X19" s="46" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="Y19" s="46" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Z19" s="46" t="s">
-        <v>153</v>
-      </c>
-      <c r="AA19" s="46" t="s">
         <v>154</v>
       </c>
+      <c r="AB19" s="46" t="s">
+        <v>172</v>
+      </c>
       <c r="AC19" s="46" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AD19" s="46" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AE19" s="46" t="s">
-        <v>174</v>
-      </c>
-      <c r="AF19" s="46" t="s">
         <v>171</v>
       </c>
-      <c r="AH19" s="51" t="s">
+      <c r="AG19" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="AI19" s="51" t="s">
+      <c r="AH19" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="AJ19" s="51" t="s">
+      <c r="AI19" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="AK19" s="51" t="s">
+      <c r="AJ19" s="50" t="s">
         <v>161</v>
       </c>
+      <c r="AM19" s="46" t="s">
+        <v>155</v>
+      </c>
       <c r="AN19" s="46" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AO19" s="46" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AP19" s="46" t="s">
-        <v>157</v>
-      </c>
-      <c r="AQ19" s="46" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="21" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="21" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N21" s="46" t="s">
         <v>158</v>
       </c>
-      <c r="O21" s="48" t="s">
+      <c r="O21" s="73" t="s">
         <v>178</v>
       </c>
-      <c r="P21" s="48" t="s">
+      <c r="P21" s="73" t="s">
         <v>170</v>
       </c>
-      <c r="Q21" s="48"/>
-      <c r="R21" s="48" t="s">
+      <c r="Q21" s="73"/>
+      <c r="R21" s="73" t="s">
         <v>182</v>
       </c>
-      <c r="S21" s="48" t="s">
+      <c r="S21" s="73" t="s">
         <v>195</v>
       </c>
-      <c r="T21" s="48"/>
-      <c r="X21" s="56" t="s">
+      <c r="W21" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="Y21" s="56" t="s">
+      <c r="X21" s="55" t="s">
         <v>201</v>
       </c>
-      <c r="Z21" s="56" t="s">
+      <c r="Y21" s="55" t="s">
         <v>200</v>
       </c>
-      <c r="AA21" s="56" t="s">
+      <c r="Z21" s="55" t="s">
         <v>199</v>
       </c>
-      <c r="AB21" s="32"/>
-      <c r="AC21" s="53" t="s">
+      <c r="AA21" s="32"/>
+      <c r="AB21" s="52" t="s">
         <v>187</v>
       </c>
-      <c r="AD21" s="53" t="s">
-        <v>10</v>
-      </c>
-      <c r="AE21" s="53" t="s">
+      <c r="AC21" s="52" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD21" s="52" t="s">
         <v>193</v>
       </c>
-      <c r="AF21" s="53" t="s">
+      <c r="AE21" s="52" t="s">
         <v>192</v>
       </c>
+      <c r="AG21" s="32">
+        <v>0</v>
+      </c>
       <c r="AH21" s="32">
         <v>0</v>
       </c>
@@ -9300,12 +9298,12 @@
       <c r="AJ21" s="32">
         <v>0</v>
       </c>
-      <c r="AK21" s="32">
-        <v>0</v>
-      </c>
-      <c r="AL21" s="52" t="s">
+      <c r="AK21" s="51" t="s">
         <v>162</v>
       </c>
+      <c r="AM21" s="32">
+        <v>0</v>
+      </c>
       <c r="AN21" s="32">
         <v>0</v>
       </c>
@@ -9315,42 +9313,41 @@
       <c r="AP21" s="32">
         <v>0</v>
       </c>
-      <c r="AQ21" s="32">
-        <v>0</v>
-      </c>
-      <c r="AR21" s="55" t="s">
+      <c r="AQ21" s="54" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="22" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="22" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N22" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="O22" s="48" t="s">
+      <c r="O22" s="73" t="s">
         <v>177</v>
       </c>
-      <c r="P22" s="48" t="s">
+      <c r="P22" s="73" t="s">
         <v>169</v>
       </c>
-      <c r="Q22" s="48"/>
-      <c r="R22" s="48" t="s">
+      <c r="Q22" s="73"/>
+      <c r="R22" s="73" t="s">
         <v>166</v>
       </c>
-      <c r="S22" s="48" t="s">
+      <c r="S22" s="73" t="s">
         <v>164</v>
       </c>
-      <c r="T22" s="48"/>
-      <c r="X22" s="73" t="s">
+      <c r="W22" s="68" t="s">
         <v>203</v>
       </c>
-      <c r="Y22" s="73"/>
-      <c r="Z22" s="73"/>
-      <c r="AA22" s="73"/>
+      <c r="X22" s="68"/>
+      <c r="Y22" s="68"/>
+      <c r="Z22" s="68"/>
+      <c r="AA22" s="32"/>
       <c r="AB22" s="32"/>
       <c r="AC22" s="32"/>
       <c r="AD22" s="32"/>
       <c r="AE22" s="32"/>
-      <c r="AF22" s="32"/>
+      <c r="AG22" s="32">
+        <v>0</v>
+      </c>
       <c r="AH22" s="32">
         <v>0</v>
       </c>
@@ -9358,14 +9355,14 @@
         <v>0</v>
       </c>
       <c r="AJ22" s="32">
-        <v>0</v>
-      </c>
-      <c r="AK22" s="32">
-        <v>1</v>
-      </c>
-      <c r="AL22" s="52" t="s">
+        <v>1</v>
+      </c>
+      <c r="AK22" s="51" t="s">
         <v>163</v>
       </c>
+      <c r="AM22" s="32">
+        <v>0</v>
+      </c>
       <c r="AN22" s="32">
         <v>0</v>
       </c>
@@ -9373,264 +9370,262 @@
         <v>0</v>
       </c>
       <c r="AP22" s="32">
-        <v>0</v>
-      </c>
-      <c r="AQ22" s="32">
-        <v>1</v>
-      </c>
-      <c r="AR22" s="55" t="s">
+        <v>1</v>
+      </c>
+      <c r="AQ22" s="54" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="23" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="23" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N23" s="46" t="s">
         <v>160</v>
       </c>
-      <c r="O23" s="48" t="s">
+      <c r="O23" s="73" t="s">
         <v>176</v>
       </c>
-      <c r="P23" s="48" t="s">
+      <c r="P23" s="73" t="s">
         <v>168</v>
       </c>
-      <c r="Q23" s="48" t="s">
+      <c r="Q23" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="R23" s="48" t="s">
+      <c r="R23" s="73" t="s">
         <v>165</v>
       </c>
-      <c r="S23" s="48" t="s">
+      <c r="S23" s="73" t="s">
         <v>163</v>
       </c>
-      <c r="T23" s="48"/>
+      <c r="AA23" s="32"/>
       <c r="AB23" s="32"/>
       <c r="AC23" s="32"/>
       <c r="AD23" s="32"/>
       <c r="AE23" s="32"/>
-      <c r="AF23" s="32"/>
+      <c r="AG23" s="32">
+        <v>0</v>
+      </c>
       <c r="AH23" s="32">
         <v>0</v>
       </c>
       <c r="AI23" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ23" s="32">
-        <v>1</v>
-      </c>
-      <c r="AK23" s="32">
-        <v>0</v>
-      </c>
-      <c r="AL23" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="AK23" s="51" t="s">
         <v>164</v>
       </c>
+      <c r="AM23" s="32">
+        <v>0</v>
+      </c>
       <c r="AN23" s="32">
         <v>0</v>
       </c>
       <c r="AO23" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP23" s="32">
-        <v>1</v>
-      </c>
-      <c r="AQ23" s="32">
-        <v>0</v>
-      </c>
-      <c r="AR23" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ23" s="54" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="24" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="24" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N24" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="O24" s="48" t="s">
+      <c r="O24" s="73" t="s">
         <v>175</v>
       </c>
-      <c r="P24" s="48" t="s">
+      <c r="P24" s="73" t="s">
         <v>167</v>
       </c>
-      <c r="Q24" s="48" t="s">
+      <c r="Q24" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="R24" s="48" t="s">
+      <c r="R24" s="73" t="s">
         <v>196</v>
       </c>
-      <c r="S24" s="48" t="s">
+      <c r="S24" s="73" t="s">
         <v>162</v>
       </c>
-      <c r="T24" s="48"/>
+      <c r="AA24" s="32"/>
       <c r="AB24" s="32"/>
       <c r="AC24" s="32"/>
       <c r="AD24" s="32"/>
       <c r="AE24" s="32"/>
-      <c r="AF24" s="32"/>
+      <c r="AG24" s="32">
+        <v>0</v>
+      </c>
       <c r="AH24" s="32">
         <v>0</v>
       </c>
       <c r="AI24" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ24" s="32">
         <v>1</v>
       </c>
-      <c r="AK24" s="32">
-        <v>1</v>
-      </c>
-      <c r="AL24" s="52" t="s">
+      <c r="AK24" s="51" t="s">
         <v>195</v>
       </c>
+      <c r="AM24" s="32">
+        <v>0</v>
+      </c>
       <c r="AN24" s="32">
         <v>0</v>
       </c>
       <c r="AO24" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP24" s="32">
         <v>1</v>
       </c>
-      <c r="AQ24" s="32">
-        <v>1</v>
-      </c>
-      <c r="AR24" s="55" t="s">
+      <c r="AQ24" s="54" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="25" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="25" spans="14:43" x14ac:dyDescent="0.25">
+      <c r="AA25" s="32"/>
       <c r="AB25" s="32"/>
       <c r="AC25" s="32"/>
       <c r="AD25" s="32"/>
       <c r="AE25" s="32"/>
-      <c r="AF25" s="32"/>
+      <c r="AG25" s="32">
+        <v>0</v>
+      </c>
       <c r="AH25" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI25" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ25" s="32">
         <v>0</v>
       </c>
-      <c r="AK25" s="32">
-        <v>0</v>
-      </c>
-      <c r="AL25" s="52" t="s">
+      <c r="AK25" s="51" t="s">
         <v>196</v>
       </c>
+      <c r="AM25" s="32">
+        <v>0</v>
+      </c>
       <c r="AN25" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO25" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP25" s="32">
         <v>0</v>
       </c>
-      <c r="AQ25" s="32">
-        <v>0</v>
-      </c>
-      <c r="AR25" s="55" t="s">
+      <c r="AQ25" s="54" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="26" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N26" s="46" t="s">
         <v>172</v>
       </c>
-      <c r="V26" s="49" t="s">
+      <c r="U26" s="48" t="s">
         <v>170</v>
       </c>
+      <c r="AA26" s="32"/>
       <c r="AB26" s="32"/>
       <c r="AC26" s="32"/>
       <c r="AD26" s="32"/>
       <c r="AE26" s="32"/>
-      <c r="AF26" s="32"/>
+      <c r="AG26" s="32">
+        <v>0</v>
+      </c>
       <c r="AH26" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI26" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ26" s="32">
-        <v>0</v>
-      </c>
-      <c r="AK26" s="32">
-        <v>1</v>
-      </c>
-      <c r="AL26" s="52" t="s">
+        <v>1</v>
+      </c>
+      <c r="AK26" s="51" t="s">
         <v>165</v>
       </c>
+      <c r="AM26" s="32">
+        <v>0</v>
+      </c>
       <c r="AN26" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO26" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP26" s="32">
-        <v>0</v>
-      </c>
-      <c r="AQ26" s="32">
-        <v>1</v>
-      </c>
-      <c r="AR26" s="55" t="s">
+        <v>1</v>
+      </c>
+      <c r="AQ26" s="54" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="27" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N27" s="46" t="s">
         <v>173</v>
       </c>
-      <c r="V27" s="52" t="s">
+      <c r="U27" s="51" t="s">
         <v>194</v>
       </c>
+      <c r="AA27" s="32"/>
       <c r="AB27" s="32"/>
       <c r="AC27" s="32"/>
       <c r="AD27" s="32"/>
       <c r="AE27" s="32"/>
-      <c r="AF27" s="32"/>
+      <c r="AG27" s="32">
+        <v>0</v>
+      </c>
       <c r="AH27" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI27" s="32">
         <v>1</v>
       </c>
       <c r="AJ27" s="32">
-        <v>1</v>
-      </c>
-      <c r="AK27" s="32">
-        <v>0</v>
-      </c>
-      <c r="AL27" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="AK27" s="51" t="s">
         <v>166</v>
       </c>
+      <c r="AM27" s="32">
+        <v>0</v>
+      </c>
       <c r="AN27" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO27" s="32">
         <v>1</v>
       </c>
       <c r="AP27" s="32">
-        <v>1</v>
-      </c>
-      <c r="AQ27" s="32">
-        <v>0</v>
-      </c>
-      <c r="AR27" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="AQ27" s="54" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="28" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="28" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N28" s="46" t="s">
         <v>174</v>
       </c>
-      <c r="V28" s="49" t="s">
+      <c r="U28" s="48" t="s">
         <v>175</v>
       </c>
-      <c r="AB28" s="32"/>
-      <c r="AC28" s="50"/>
-      <c r="AD28" s="50"/>
-      <c r="AE28" s="50"/>
-      <c r="AF28" s="50"/>
+      <c r="AA28" s="32"/>
+      <c r="AB28" s="49"/>
+      <c r="AC28" s="49"/>
+      <c r="AD28" s="49"/>
+      <c r="AE28" s="49"/>
+      <c r="AG28" s="32">
+        <v>0</v>
+      </c>
       <c r="AH28" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI28" s="32">
         <v>1</v>
@@ -9638,39 +9633,39 @@
       <c r="AJ28" s="32">
         <v>1</v>
       </c>
-      <c r="AK28" s="32">
-        <v>1</v>
-      </c>
-      <c r="AL28" s="52" t="s">
+      <c r="AK28" s="51" t="s">
         <v>182</v>
       </c>
-      <c r="AN28" s="50">
-        <v>0</v>
-      </c>
-      <c r="AO28" s="50">
-        <v>1</v>
-      </c>
-      <c r="AP28" s="50">
-        <v>1</v>
-      </c>
-      <c r="AQ28" s="50">
-        <v>1</v>
-      </c>
-      <c r="AR28" t="s">
+      <c r="AM28" s="49">
+        <v>0</v>
+      </c>
+      <c r="AN28" s="49">
+        <v>1</v>
+      </c>
+      <c r="AO28" s="49">
+        <v>1</v>
+      </c>
+      <c r="AP28" s="49">
+        <v>1</v>
+      </c>
+      <c r="AQ28" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="29" spans="14:44" x14ac:dyDescent="0.25">
-      <c r="N29" s="54" t="s">
+    <row r="29" spans="14:43" x14ac:dyDescent="0.25">
+      <c r="N29" s="53" t="s">
         <v>171</v>
       </c>
+      <c r="AA29" s="32"/>
       <c r="AB29" s="32"/>
       <c r="AC29" s="32"/>
       <c r="AD29" s="32"/>
       <c r="AE29" s="32"/>
-      <c r="AF29" s="32"/>
+      <c r="AG29" s="32">
+        <v>1</v>
+      </c>
       <c r="AH29" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI29" s="32">
         <v>0</v>
@@ -9678,14 +9673,14 @@
       <c r="AJ29" s="32">
         <v>0</v>
       </c>
-      <c r="AK29" s="32">
-        <v>0</v>
-      </c>
-      <c r="AL29" s="52" t="s">
+      <c r="AK29" s="51" t="s">
         <v>43</v>
       </c>
+      <c r="AM29" s="32">
+        <v>1</v>
+      </c>
       <c r="AN29" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO29" s="32">
         <v>0</v>
@@ -9693,311 +9688,307 @@
       <c r="AP29" s="32">
         <v>0</v>
       </c>
-      <c r="AQ29" s="32">
-        <v>0</v>
-      </c>
-      <c r="AR29" s="55" t="s">
+      <c r="AQ29" s="54" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="30" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="30" spans="14:43" x14ac:dyDescent="0.25">
+      <c r="AA30" s="32"/>
       <c r="AB30" s="32"/>
       <c r="AC30" s="32"/>
       <c r="AD30" s="32"/>
       <c r="AE30" s="32"/>
-      <c r="AF30" s="32"/>
+      <c r="AG30" s="32">
+        <v>1</v>
+      </c>
       <c r="AH30" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI30" s="32">
         <v>0</v>
       </c>
       <c r="AJ30" s="32">
-        <v>0</v>
-      </c>
-      <c r="AK30" s="32">
-        <v>1</v>
-      </c>
-      <c r="AL30" s="52" t="s">
+        <v>1</v>
+      </c>
+      <c r="AK30" s="51" t="s">
         <v>67</v>
       </c>
+      <c r="AM30" s="32">
+        <v>1</v>
+      </c>
       <c r="AN30" s="32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO30" s="32">
         <v>0</v>
       </c>
       <c r="AP30" s="32">
-        <v>0</v>
-      </c>
-      <c r="AQ30" s="32">
-        <v>1</v>
-      </c>
-      <c r="AR30" s="55" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="31" spans="14:44" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="AQ30" s="54" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N31" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="V31" s="49" t="s">
+      <c r="U31" s="48" t="s">
         <v>178</v>
       </c>
-      <c r="AB31" s="32"/>
-      <c r="AC31" s="50"/>
-      <c r="AD31" s="50"/>
-      <c r="AE31" s="50"/>
-      <c r="AF31" s="50"/>
-      <c r="AH31" s="50">
-        <v>1</v>
-      </c>
-      <c r="AI31" s="50">
-        <v>0</v>
-      </c>
-      <c r="AJ31" s="50">
-        <v>1</v>
-      </c>
-      <c r="AK31" s="50">
-        <v>0</v>
-      </c>
-      <c r="AL31" t="s">
+      <c r="AA31" s="32"/>
+      <c r="AB31" s="49"/>
+      <c r="AC31" s="49"/>
+      <c r="AD31" s="49"/>
+      <c r="AE31" s="49"/>
+      <c r="AG31" s="49">
+        <v>1</v>
+      </c>
+      <c r="AH31" s="49">
+        <v>0</v>
+      </c>
+      <c r="AI31" s="49">
+        <v>1</v>
+      </c>
+      <c r="AJ31" s="49">
+        <v>0</v>
+      </c>
+      <c r="AK31" t="s">
         <v>191</v>
       </c>
-      <c r="AN31" s="50">
-        <v>1</v>
-      </c>
-      <c r="AO31" s="50">
-        <v>0</v>
-      </c>
-      <c r="AP31" s="50">
-        <v>1</v>
-      </c>
-      <c r="AQ31" s="50">
-        <v>0</v>
-      </c>
-      <c r="AR31" t="s">
+      <c r="AM31" s="49">
+        <v>1</v>
+      </c>
+      <c r="AN31" s="49">
+        <v>0</v>
+      </c>
+      <c r="AO31" s="49">
+        <v>1</v>
+      </c>
+      <c r="AP31" s="49">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="32" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="32" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N32" s="46" t="s">
         <v>152</v>
       </c>
-      <c r="V32" s="49" t="s">
+      <c r="U32" s="48" t="s">
         <v>167</v>
       </c>
-      <c r="AC32" s="50"/>
-      <c r="AD32" s="50"/>
-      <c r="AE32" s="50"/>
-      <c r="AF32" s="50"/>
-      <c r="AH32" s="50">
-        <v>1</v>
-      </c>
-      <c r="AI32" s="50">
-        <v>0</v>
-      </c>
-      <c r="AJ32" s="50">
-        <v>1</v>
-      </c>
-      <c r="AK32" s="50">
-        <v>1</v>
-      </c>
-      <c r="AL32" t="s">
+      <c r="AB32" s="49"/>
+      <c r="AC32" s="49"/>
+      <c r="AD32" s="49"/>
+      <c r="AE32" s="49"/>
+      <c r="AG32" s="49">
+        <v>1</v>
+      </c>
+      <c r="AH32" s="49">
+        <v>0</v>
+      </c>
+      <c r="AI32" s="49">
+        <v>1</v>
+      </c>
+      <c r="AJ32" s="49">
+        <v>1</v>
+      </c>
+      <c r="AK32" t="s">
         <v>191</v>
       </c>
-      <c r="AN32" s="50">
-        <v>1</v>
-      </c>
-      <c r="AO32" s="50">
-        <v>0</v>
-      </c>
-      <c r="AP32" s="50">
-        <v>1</v>
-      </c>
-      <c r="AQ32" s="50">
-        <v>1</v>
-      </c>
-      <c r="AR32" t="s">
+      <c r="AM32" s="49">
+        <v>1</v>
+      </c>
+      <c r="AN32" s="49">
+        <v>0</v>
+      </c>
+      <c r="AO32" s="49">
+        <v>1</v>
+      </c>
+      <c r="AP32" s="49">
+        <v>1</v>
+      </c>
+      <c r="AQ32" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="33" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="33" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N33" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="V33" s="49" t="s">
+      <c r="U33" s="48" t="s">
         <v>168</v>
       </c>
-      <c r="AC33" s="50"/>
-      <c r="AD33" s="50"/>
-      <c r="AE33" s="50"/>
-      <c r="AF33" s="50"/>
-      <c r="AH33" s="50">
-        <v>1</v>
-      </c>
-      <c r="AI33" s="50">
-        <v>1</v>
-      </c>
-      <c r="AJ33" s="50">
-        <v>0</v>
-      </c>
-      <c r="AK33" s="50">
-        <v>0</v>
-      </c>
-      <c r="AL33" t="s">
+      <c r="AB33" s="49"/>
+      <c r="AC33" s="49"/>
+      <c r="AD33" s="49"/>
+      <c r="AE33" s="49"/>
+      <c r="AG33" s="49">
+        <v>1</v>
+      </c>
+      <c r="AH33" s="49">
+        <v>1</v>
+      </c>
+      <c r="AI33" s="49">
+        <v>0</v>
+      </c>
+      <c r="AJ33" s="49">
+        <v>0</v>
+      </c>
+      <c r="AK33" t="s">
         <v>191</v>
       </c>
-      <c r="AN33" s="50">
-        <v>1</v>
-      </c>
-      <c r="AO33" s="50">
-        <v>1</v>
-      </c>
-      <c r="AP33" s="50">
-        <v>0</v>
-      </c>
-      <c r="AQ33" s="50">
-        <v>0</v>
-      </c>
-      <c r="AR33" t="s">
+      <c r="AM33" s="49">
+        <v>1</v>
+      </c>
+      <c r="AN33" s="49">
+        <v>1</v>
+      </c>
+      <c r="AO33" s="49">
+        <v>0</v>
+      </c>
+      <c r="AP33" s="49">
+        <v>0</v>
+      </c>
+      <c r="AQ33" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="34" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="34" spans="14:43" x14ac:dyDescent="0.25">
       <c r="N34" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="V34" s="49" t="s">
+      <c r="U34" s="48" t="s">
         <v>169</v>
       </c>
-      <c r="AC34" s="50"/>
-      <c r="AD34" s="50"/>
-      <c r="AE34" s="50"/>
-      <c r="AF34" s="50"/>
-      <c r="AH34" s="50">
-        <v>1</v>
-      </c>
-      <c r="AI34" s="50">
-        <v>1</v>
-      </c>
-      <c r="AJ34" s="50">
-        <v>0</v>
-      </c>
-      <c r="AK34" s="50">
-        <v>1</v>
-      </c>
-      <c r="AL34" t="s">
+      <c r="AB34" s="49"/>
+      <c r="AC34" s="49"/>
+      <c r="AD34" s="49"/>
+      <c r="AE34" s="49"/>
+      <c r="AG34" s="49">
+        <v>1</v>
+      </c>
+      <c r="AH34" s="49">
+        <v>1</v>
+      </c>
+      <c r="AI34" s="49">
+        <v>0</v>
+      </c>
+      <c r="AJ34" s="49">
+        <v>1</v>
+      </c>
+      <c r="AK34" t="s">
         <v>191</v>
       </c>
-      <c r="AN34" s="50">
-        <v>1</v>
-      </c>
-      <c r="AO34" s="50">
-        <v>1</v>
-      </c>
-      <c r="AP34" s="50">
-        <v>0</v>
-      </c>
-      <c r="AQ34" s="50">
-        <v>1</v>
-      </c>
-      <c r="AR34" t="s">
+      <c r="AM34" s="49">
+        <v>1</v>
+      </c>
+      <c r="AN34" s="49">
+        <v>1</v>
+      </c>
+      <c r="AO34" s="49">
+        <v>0</v>
+      </c>
+      <c r="AP34" s="49">
+        <v>1</v>
+      </c>
+      <c r="AQ34" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="35" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="35" spans="14:43" x14ac:dyDescent="0.25">
       <c r="P35" s="32"/>
       <c r="Q35" s="32"/>
       <c r="R35" s="32"/>
       <c r="S35" s="32"/>
       <c r="T35" s="32"/>
-      <c r="U35" s="32"/>
-      <c r="AC35" s="50"/>
-      <c r="AD35" s="50"/>
-      <c r="AE35" s="50"/>
-      <c r="AF35" s="50"/>
-      <c r="AH35" s="50">
-        <v>1</v>
-      </c>
-      <c r="AI35" s="50">
-        <v>1</v>
-      </c>
-      <c r="AJ35" s="50">
-        <v>1</v>
-      </c>
-      <c r="AK35" s="50">
-        <v>0</v>
-      </c>
-      <c r="AL35" t="s">
+      <c r="AB35" s="49"/>
+      <c r="AC35" s="49"/>
+      <c r="AD35" s="49"/>
+      <c r="AE35" s="49"/>
+      <c r="AG35" s="49">
+        <v>1</v>
+      </c>
+      <c r="AH35" s="49">
+        <v>1</v>
+      </c>
+      <c r="AI35" s="49">
+        <v>1</v>
+      </c>
+      <c r="AJ35" s="49">
+        <v>0</v>
+      </c>
+      <c r="AK35" t="s">
         <v>191</v>
       </c>
-      <c r="AN35" s="50">
-        <v>1</v>
-      </c>
-      <c r="AO35" s="50">
-        <v>1</v>
-      </c>
-      <c r="AP35" s="50">
-        <v>1</v>
-      </c>
-      <c r="AQ35" s="50">
-        <v>0</v>
-      </c>
-      <c r="AR35" t="s">
+      <c r="AM35" s="49">
+        <v>1</v>
+      </c>
+      <c r="AN35" s="49">
+        <v>1</v>
+      </c>
+      <c r="AO35" s="49">
+        <v>1</v>
+      </c>
+      <c r="AP35" s="49">
+        <v>0</v>
+      </c>
+      <c r="AQ35" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="36" spans="14:44" x14ac:dyDescent="0.25">
+    <row r="36" spans="14:43" x14ac:dyDescent="0.25">
       <c r="S36" s="32"/>
-      <c r="U36" s="32"/>
-      <c r="AC36" s="50"/>
-      <c r="AD36" s="50"/>
-      <c r="AE36" s="50"/>
-      <c r="AF36" s="50"/>
-      <c r="AH36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AI36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AJ36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AK36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AL36" t="s">
+      <c r="T36" s="32"/>
+      <c r="AB36" s="49"/>
+      <c r="AC36" s="49"/>
+      <c r="AD36" s="49"/>
+      <c r="AE36" s="49"/>
+      <c r="AG36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AH36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AI36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AJ36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AK36" t="s">
         <v>191</v>
       </c>
-      <c r="AN36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AO36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AP36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AQ36" s="50">
-        <v>1</v>
-      </c>
-      <c r="AR36" t="s">
+      <c r="AM36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AN36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AO36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AP36" s="49">
+        <v>1</v>
+      </c>
+      <c r="AQ36" t="s">
         <v>191</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="X22:AA22"/>
+    <mergeCell ref="B2:AQ2"/>
+    <mergeCell ref="W18:AQ18"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="W22:Z22"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="N3:S3"/>
-    <mergeCell ref="O18:V18"/>
+    <mergeCell ref="O18:U18"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B2:AR2"/>
-    <mergeCell ref="X18:AR18"/>
-    <mergeCell ref="X13:Z13"/>
-    <mergeCell ref="X14:Z14"/>
-    <mergeCell ref="X15:Z15"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">
@@ -10026,33 +10017,33 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B7" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B8" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -10085,7 +10076,7 @@
         <v>106</v>
       </c>
       <c r="E3" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -10093,10 +10084,10 @@
         <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E4" s="42" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -10116,7 +10107,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G8" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>212</v>
@@ -10127,34 +10118,37 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G9" t="s">
-        <v>244</v>
-      </c>
-      <c r="I9" s="58" t="s">
+        <v>256</v>
+      </c>
+      <c r="I9" s="57" t="s">
         <v>213</v>
       </c>
       <c r="J9" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I10" s="60" t="s">
+      <c r="I10" s="59" t="s">
         <v>209</v>
       </c>
       <c r="J10" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I11" s="60" t="s">
+      <c r="I11" s="59" t="s">
         <v>214</v>
       </c>
       <c r="J11" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I12" s="59" t="s">
+      <c r="I12" s="58" t="s">
         <v>215</v>
+      </c>
+      <c r="J12" s="42" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -10162,10 +10156,10 @@
         <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E13" s="42" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -10183,7 +10177,7 @@
         <v>208</v>
       </c>
       <c r="J16" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
@@ -10212,7 +10206,7 @@
       <c r="G19" t="s">
         <v>217</v>
       </c>
-      <c r="I19" s="58" t="s">
+      <c r="I19" s="57" t="s">
         <v>209</v>
       </c>
       <c r="J19" t="s">
@@ -10220,7 +10214,7 @@
       </c>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I20" s="59" t="s">
+      <c r="I20" s="58" t="s">
         <v>214</v>
       </c>
     </row>
@@ -10239,9 +10233,6 @@
         <v>76</v>
       </c>
       <c r="E23" s="42"/>
-      <c r="G23" t="s">
-        <v>227</v>
-      </c>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
       <c r="E24">
@@ -10259,7 +10250,7 @@
         <v>207</v>
       </c>
       <c r="K25" t="s">
-        <v>225</v>
+        <v>255</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
@@ -10352,7 +10343,7 @@
       <c r="E37">
         <v>0</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I37" s="9" t="s">
         <v>213</v>
       </c>
     </row>
@@ -10385,7 +10376,7 @@
         <v>78</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.25">
@@ -10398,7 +10389,7 @@
         <v>80</v>
       </c>
       <c r="K43" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="44" spans="2:11" x14ac:dyDescent="0.25">
@@ -10425,51 +10416,51 @@
       </c>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B48" s="58" t="s">
+      <c r="B48" s="57" t="s">
         <v>95</v>
       </c>
       <c r="C48" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="G48" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B49" s="60" t="s">
+      <c r="B49" s="59" t="s">
         <v>96</v>
       </c>
       <c r="D49" t="s">
         <v>220</v>
       </c>
       <c r="G49" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B50" s="60" t="s">
+      <c r="B50" s="59" t="s">
         <v>97</v>
       </c>
       <c r="G50" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B51" s="59" t="s">
+      <c r="B51" s="58" t="s">
         <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="D51" t="s">
         <v>221</v>
       </c>
       <c r="G51" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B52" s="58" t="s">
+      <c r="B52" s="57" t="s">
         <v>83</v>
       </c>
       <c r="E52" t="s">
@@ -10477,7 +10468,7 @@
       </c>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B53" s="60" t="s">
+      <c r="B53" s="59" t="s">
         <v>84</v>
       </c>
       <c r="D53" t="s">
@@ -10488,7 +10479,7 @@
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" s="60" t="s">
+      <c r="B54" s="59" t="s">
         <v>85</v>
       </c>
       <c r="E54" t="s">
@@ -10496,7 +10487,7 @@
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" s="59" t="s">
+      <c r="B55" s="58" t="s">
         <v>86</v>
       </c>
       <c r="D55" t="s">
@@ -10507,7 +10498,7 @@
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" s="58" t="s">
+      <c r="B56" s="57" t="s">
         <v>87</v>
       </c>
       <c r="E56" t="s">
@@ -10515,21 +10506,21 @@
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="60" t="s">
+      <c r="B57" s="59" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="60" t="s">
+      <c r="B58" s="59" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="59" t="s">
+      <c r="B59" s="58" t="s">
         <v>90</v>
       </c>
       <c r="K59" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.25">
@@ -10537,7 +10528,7 @@
         <v>91</v>
       </c>
       <c r="E60" s="42" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
@@ -10545,7 +10536,7 @@
         <v>92</v>
       </c>
       <c r="E61" s="42" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
@@ -10561,7 +10552,7 @@
         <v>100</v>
       </c>
       <c r="E63" s="42" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
@@ -10569,7 +10560,7 @@
         <v>101</v>
       </c>
       <c r="E64" s="42" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
@@ -10577,7 +10568,7 @@
         <v>102</v>
       </c>
       <c r="E65" s="42" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
@@ -10606,22 +10597,22 @@
   <sheetData>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C3" t="s">
+        <v>226</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>228</v>
+      </c>
+      <c r="E3" t="s">
         <v>229</v>
       </c>
-      <c r="C3" t="s">
-        <v>228</v>
-      </c>
-      <c r="D3" s="42" t="s">
+      <c r="F3" t="s">
         <v>230</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>231</v>
-      </c>
-      <c r="F3" t="s">
-        <v>232</v>
-      </c>
-      <c r="G3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added LA-traces, some assembly-comments
</commit_message>
<xml_diff>
--- a/Data/PM2528 Technical details.xlsx
+++ b/Data/PM2528 Technical details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B668C8F4-C42D-4347-9A42-9203E1C22721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B844BA-C7E4-4630-A2E2-C84F5A7459E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
+    <workbookView xWindow="-28695" yWindow="7815" windowWidth="28800" windowHeight="13065" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
   <sheets>
     <sheet name="MainBoard-Relais" sheetId="3" r:id="rId1"/>
@@ -824,7 +824,7 @@
     <t>0000=VDC, 0001=VAC, 0010=VDCAC, 0011=R2W</t>
   </si>
   <si>
-    <t>00100=R4W, 00101ADC, 0110=ADCAC, 0111=C</t>
+    <t>0100=R4W, 0101ADC, 0110=ADCAC, 0111=C</t>
   </si>
 </sst>
 </file>
@@ -1304,6 +1304,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1328,11 +1329,11 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1340,10 +1341,9 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1710,78 +1710,78 @@
       <c r="BE1" s="3"/>
     </row>
     <row r="2" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="C2" s="60" t="s">
+      <c r="C2" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="60" t="s">
+      <c r="I2" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="60"/>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="60"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="M2" s="61"/>
       <c r="N2" s="3"/>
-      <c r="O2" s="60" t="s">
+      <c r="O2" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="P2" s="60"/>
-      <c r="Q2" s="60"/>
-      <c r="R2" s="60"/>
-      <c r="S2" s="60"/>
+      <c r="P2" s="61"/>
+      <c r="Q2" s="61"/>
+      <c r="R2" s="61"/>
+      <c r="S2" s="61"/>
       <c r="T2" s="3"/>
-      <c r="U2" s="60" t="s">
+      <c r="U2" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="V2" s="60"/>
-      <c r="W2" s="60"/>
-      <c r="X2" s="60"/>
-      <c r="Y2" s="60"/>
-      <c r="Z2" s="60"/>
-      <c r="AA2" s="60"/>
-      <c r="AB2" s="60"/>
+      <c r="V2" s="61"/>
+      <c r="W2" s="61"/>
+      <c r="X2" s="61"/>
+      <c r="Y2" s="61"/>
+      <c r="Z2" s="61"/>
+      <c r="AA2" s="61"/>
+      <c r="AB2" s="61"/>
       <c r="AC2" s="3"/>
-      <c r="AD2" s="60" t="s">
+      <c r="AD2" s="61" t="s">
         <v>34</v>
       </c>
-      <c r="AE2" s="60"/>
-      <c r="AF2" s="60"/>
-      <c r="AG2" s="60"/>
-      <c r="AH2" s="60"/>
+      <c r="AE2" s="61"/>
+      <c r="AF2" s="61"/>
+      <c r="AG2" s="61"/>
+      <c r="AH2" s="61"/>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="60" t="s">
+      <c r="AJ2" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="AK2" s="60"/>
-      <c r="AL2" s="60"/>
-      <c r="AM2" s="60"/>
-      <c r="AN2" s="60"/>
-      <c r="AO2" s="60"/>
-      <c r="AP2" s="60"/>
+      <c r="AK2" s="61"/>
+      <c r="AL2" s="61"/>
+      <c r="AM2" s="61"/>
+      <c r="AN2" s="61"/>
+      <c r="AO2" s="61"/>
+      <c r="AP2" s="61"/>
       <c r="AQ2" s="3"/>
-      <c r="AR2" s="60" t="s">
+      <c r="AR2" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="AS2" s="60"/>
-      <c r="AT2" s="60"/>
-      <c r="AU2" s="60"/>
-      <c r="AV2" s="60"/>
-      <c r="AW2" s="60"/>
-      <c r="AX2" s="60"/>
+      <c r="AS2" s="61"/>
+      <c r="AT2" s="61"/>
+      <c r="AU2" s="61"/>
+      <c r="AV2" s="61"/>
+      <c r="AW2" s="61"/>
+      <c r="AX2" s="61"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="BA2" s="3"/>
-      <c r="BB2" s="60" t="s">
+      <c r="BB2" s="61" t="s">
         <v>67</v>
       </c>
-      <c r="BC2" s="60"/>
-      <c r="BD2" s="60"/>
+      <c r="BC2" s="61"/>
+      <c r="BD2" s="61"/>
       <c r="BE2" s="3"/>
       <c r="BF2" s="41" t="s">
         <v>43</v>
@@ -7000,69 +7000,69 @@
       </c>
     </row>
     <row r="2" spans="1:29" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D2" s="63" t="s">
+      <c r="D2" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="63"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="63"/>
-      <c r="L2" s="63"/>
-      <c r="M2" s="63"/>
-      <c r="N2" s="63"/>
-      <c r="O2" s="63"/>
-      <c r="P2" s="63"/>
-      <c r="Q2" s="63"/>
-      <c r="R2" s="63"/>
-      <c r="S2" s="63"/>
-      <c r="T2" s="63"/>
-      <c r="U2" s="63"/>
-      <c r="V2" s="63"/>
-      <c r="W2" s="63"/>
-      <c r="X2" s="63"/>
-      <c r="Y2" s="63"/>
-      <c r="Z2" s="63"/>
-      <c r="AA2" s="63"/>
-      <c r="AB2" s="63"/>
-      <c r="AC2" s="63"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="64"/>
+      <c r="P2" s="64"/>
+      <c r="Q2" s="64"/>
+      <c r="R2" s="64"/>
+      <c r="S2" s="64"/>
+      <c r="T2" s="64"/>
+      <c r="U2" s="64"/>
+      <c r="V2" s="64"/>
+      <c r="W2" s="64"/>
+      <c r="X2" s="64"/>
+      <c r="Y2" s="64"/>
+      <c r="Z2" s="64"/>
+      <c r="AA2" s="64"/>
+      <c r="AB2" s="64"/>
+      <c r="AC2" s="64"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="D3" s="64" t="s">
+      <c r="D3" s="65" t="s">
         <v>135</v>
       </c>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="62"/>
-      <c r="N3" s="65" t="s">
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="63"/>
+      <c r="N3" s="66" t="s">
         <v>113</v>
       </c>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="66"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
       <c r="R3" s="18"/>
-      <c r="S3" s="66" t="s">
+      <c r="S3" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="T3" s="66"/>
-      <c r="U3" s="66"/>
-      <c r="V3" s="67"/>
-      <c r="X3" s="64" t="s">
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="68"/>
+      <c r="X3" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="Y3" s="61"/>
-      <c r="Z3" s="61"/>
+      <c r="Y3" s="62"/>
+      <c r="Z3" s="62"/>
       <c r="AA3" s="17"/>
-      <c r="AB3" s="61" t="s">
+      <c r="AB3" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="AC3" s="62"/>
+      <c r="AC3" s="63"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="D4" s="22" t="s">
@@ -8557,50 +8557,50 @@
       <c r="T1" s="32"/>
     </row>
     <row r="2" spans="2:43" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="64" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="63"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="63"/>
-      <c r="L2" s="63"/>
-      <c r="M2" s="63"/>
-      <c r="N2" s="63"/>
-      <c r="O2" s="63"/>
-      <c r="P2" s="63"/>
-      <c r="Q2" s="63"/>
-      <c r="R2" s="63"/>
-      <c r="S2" s="63"/>
-      <c r="T2" s="63"/>
-      <c r="U2" s="63"/>
-      <c r="V2" s="63"/>
-      <c r="W2" s="63"/>
-      <c r="X2" s="63"/>
-      <c r="Y2" s="63"/>
-      <c r="Z2" s="63"/>
-      <c r="AA2" s="63"/>
-      <c r="AB2" s="63"/>
-      <c r="AC2" s="63"/>
-      <c r="AD2" s="63"/>
-      <c r="AE2" s="63"/>
-      <c r="AF2" s="63"/>
-      <c r="AG2" s="63"/>
-      <c r="AH2" s="63"/>
-      <c r="AI2" s="63"/>
-      <c r="AJ2" s="63"/>
-      <c r="AK2" s="63"/>
-      <c r="AL2" s="63"/>
-      <c r="AM2" s="63"/>
-      <c r="AN2" s="63"/>
-      <c r="AO2" s="63"/>
-      <c r="AP2" s="63"/>
-      <c r="AQ2" s="63"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="64"/>
+      <c r="P2" s="64"/>
+      <c r="Q2" s="64"/>
+      <c r="R2" s="64"/>
+      <c r="S2" s="64"/>
+      <c r="T2" s="64"/>
+      <c r="U2" s="64"/>
+      <c r="V2" s="64"/>
+      <c r="W2" s="64"/>
+      <c r="X2" s="64"/>
+      <c r="Y2" s="64"/>
+      <c r="Z2" s="64"/>
+      <c r="AA2" s="64"/>
+      <c r="AB2" s="64"/>
+      <c r="AC2" s="64"/>
+      <c r="AD2" s="64"/>
+      <c r="AE2" s="64"/>
+      <c r="AF2" s="64"/>
+      <c r="AG2" s="64"/>
+      <c r="AH2" s="64"/>
+      <c r="AI2" s="64"/>
+      <c r="AJ2" s="64"/>
+      <c r="AK2" s="64"/>
+      <c r="AL2" s="64"/>
+      <c r="AM2" s="64"/>
+      <c r="AN2" s="64"/>
+      <c r="AO2" s="64"/>
+      <c r="AP2" s="64"/>
+      <c r="AQ2" s="64"/>
     </row>
     <row r="3" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B3" s="69" t="s">
@@ -9099,11 +9099,11 @@
       <c r="S13" s="55">
         <v>0</v>
       </c>
-      <c r="W13" s="72" t="s">
+      <c r="W13" s="70" t="s">
         <v>180</v>
       </c>
-      <c r="X13" s="72"/>
-      <c r="Y13" s="72"/>
+      <c r="X13" s="70"/>
+      <c r="Y13" s="70"/>
     </row>
     <row r="14" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
@@ -9112,11 +9112,11 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="W14" s="70" t="s">
+      <c r="W14" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="X14" s="70"/>
-      <c r="Y14" s="70"/>
+      <c r="X14" s="71"/>
+      <c r="Y14" s="71"/>
     </row>
     <row r="15" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
@@ -9127,11 +9127,11 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="W15" s="71" t="s">
+      <c r="W15" s="72" t="s">
         <v>198</v>
       </c>
-      <c r="X15" s="71"/>
-      <c r="Y15" s="71"/>
+      <c r="X15" s="72"/>
+      <c r="Y15" s="72"/>
     </row>
     <row r="16" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
@@ -9248,17 +9248,17 @@
       <c r="N21" s="46" t="s">
         <v>158</v>
       </c>
-      <c r="O21" s="73" t="s">
+      <c r="O21" s="60" t="s">
         <v>178</v>
       </c>
-      <c r="P21" s="73" t="s">
+      <c r="P21" s="60" t="s">
         <v>170</v>
       </c>
-      <c r="Q21" s="73"/>
-      <c r="R21" s="73" t="s">
+      <c r="Q21" s="60"/>
+      <c r="R21" s="60" t="s">
         <v>182</v>
       </c>
-      <c r="S21" s="73" t="s">
+      <c r="S21" s="60" t="s">
         <v>195</v>
       </c>
       <c r="W21" s="55" t="s">
@@ -9321,25 +9321,25 @@
       <c r="N22" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="O22" s="73" t="s">
+      <c r="O22" s="60" t="s">
         <v>177</v>
       </c>
-      <c r="P22" s="73" t="s">
+      <c r="P22" s="60" t="s">
         <v>169</v>
       </c>
-      <c r="Q22" s="73"/>
-      <c r="R22" s="73" t="s">
+      <c r="Q22" s="60"/>
+      <c r="R22" s="60" t="s">
         <v>166</v>
       </c>
-      <c r="S22" s="73" t="s">
+      <c r="S22" s="60" t="s">
         <v>164</v>
       </c>
-      <c r="W22" s="68" t="s">
+      <c r="W22" s="73" t="s">
         <v>203</v>
       </c>
-      <c r="X22" s="68"/>
-      <c r="Y22" s="68"/>
-      <c r="Z22" s="68"/>
+      <c r="X22" s="73"/>
+      <c r="Y22" s="73"/>
+      <c r="Z22" s="73"/>
       <c r="AA22" s="32"/>
       <c r="AB22" s="32"/>
       <c r="AC22" s="32"/>
@@ -9380,19 +9380,19 @@
       <c r="N23" s="46" t="s">
         <v>160</v>
       </c>
-      <c r="O23" s="73" t="s">
+      <c r="O23" s="60" t="s">
         <v>176</v>
       </c>
-      <c r="P23" s="73" t="s">
+      <c r="P23" s="60" t="s">
         <v>168</v>
       </c>
-      <c r="Q23" s="73" t="s">
+      <c r="Q23" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="R23" s="73" t="s">
+      <c r="R23" s="60" t="s">
         <v>165</v>
       </c>
-      <c r="S23" s="73" t="s">
+      <c r="S23" s="60" t="s">
         <v>163</v>
       </c>
       <c r="AA23" s="32"/>
@@ -9435,19 +9435,19 @@
       <c r="N24" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="O24" s="73" t="s">
+      <c r="O24" s="60" t="s">
         <v>175</v>
       </c>
-      <c r="P24" s="73" t="s">
+      <c r="P24" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="Q24" s="73" t="s">
+      <c r="Q24" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="R24" s="73" t="s">
+      <c r="R24" s="60" t="s">
         <v>196</v>
       </c>
-      <c r="S24" s="73" t="s">
+      <c r="S24" s="60" t="s">
         <v>162</v>
       </c>
       <c r="AA24" s="32"/>
@@ -9979,16 +9979,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="W22:Z22"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="O18:U18"/>
+    <mergeCell ref="B3:I3"/>
     <mergeCell ref="B2:AQ2"/>
     <mergeCell ref="W18:AQ18"/>
     <mergeCell ref="W13:Y13"/>
     <mergeCell ref="W14:Y14"/>
     <mergeCell ref="W15:Y15"/>
-    <mergeCell ref="W22:Z22"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="N3:S3"/>
-    <mergeCell ref="O18:U18"/>
-    <mergeCell ref="B3:I3"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">

</xml_diff>

<commit_message>
Included PCBs, Risercard and 3D-views
</commit_message>
<xml_diff>
--- a/Data/PM2528 Technical details.xlsx
+++ b/Data/PM2528 Technical details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Gadgets\Philips PM2528 DMM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B844BA-C7E4-4630-A2E2-C84F5A7459E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A8E7EFD-57F9-421A-91D5-4BD2EBEBD577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28695" yWindow="7815" windowWidth="28800" windowHeight="13065" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{1BACE0FD-08C6-41B4-8CD8-ADA47AB22099}"/>
   </bookViews>
   <sheets>
     <sheet name="MainBoard-Relais" sheetId="3" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="N2 (Display)" sheetId="7" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId4"/>
     <sheet name="InternalMemory" sheetId="6" r:id="rId5"/>
-    <sheet name="N30" sheetId="8" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'MainBoard-Relais'!$A$1:$AZ$47</definedName>
@@ -45,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1691" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="254">
   <si>
     <t>N23 (Current source)</t>
   </si>
@@ -723,24 +722,6 @@
   </si>
   <si>
     <t>1 = N30.R3019=1, Galvanic type 1</t>
-  </si>
-  <si>
-    <t>A3</t>
-  </si>
-  <si>
-    <t>A4</t>
-  </si>
-  <si>
-    <t>/WR</t>
-  </si>
-  <si>
-    <t>READ</t>
-  </si>
-  <si>
-    <t>D7</t>
-  </si>
-  <si>
-    <t>D6</t>
   </si>
   <si>
     <t>Will be written out to Extmem</t>
@@ -1329,6 +1310,9 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1340,9 +1324,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8603,29 +8584,29 @@
       <c r="AQ2" s="64"/>
     </row>
     <row r="3" spans="2:43" x14ac:dyDescent="0.25">
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="70" t="s">
         <v>204</v>
       </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="K3" s="69" t="s">
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="K3" s="70" t="s">
         <v>136</v>
       </c>
-      <c r="L3" s="69"/>
+      <c r="L3" s="70"/>
       <c r="M3" s="32"/>
-      <c r="N3" s="69" t="s">
+      <c r="N3" s="70" t="s">
         <v>137</v>
       </c>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="70"/>
+      <c r="R3" s="70"/>
+      <c r="S3" s="70"/>
     </row>
     <row r="4" spans="2:43" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
@@ -8776,7 +8757,7 @@
         <v>63</v>
       </c>
       <c r="K7" s="32" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="L7" s="32">
         <v>1</v>
@@ -9099,11 +9080,11 @@
       <c r="S13" s="55">
         <v>0</v>
       </c>
-      <c r="W13" s="70" t="s">
+      <c r="W13" s="71" t="s">
         <v>180</v>
       </c>
-      <c r="X13" s="70"/>
-      <c r="Y13" s="70"/>
+      <c r="X13" s="71"/>
+      <c r="Y13" s="71"/>
     </row>
     <row r="14" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N14" s="32"/>
@@ -9112,11 +9093,11 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
       <c r="S14" s="32"/>
-      <c r="W14" s="71" t="s">
+      <c r="W14" s="72" t="s">
         <v>197</v>
       </c>
-      <c r="X14" s="71"/>
-      <c r="Y14" s="71"/>
+      <c r="X14" s="72"/>
+      <c r="Y14" s="72"/>
     </row>
     <row r="15" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N15" s="47" t="s">
@@ -9127,11 +9108,11 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
       <c r="S15" s="32"/>
-      <c r="W15" s="72" t="s">
+      <c r="W15" s="73" t="s">
         <v>198</v>
       </c>
-      <c r="X15" s="72"/>
-      <c r="Y15" s="72"/>
+      <c r="X15" s="73"/>
+      <c r="Y15" s="73"/>
     </row>
     <row r="16" spans="2:43" x14ac:dyDescent="0.25">
       <c r="N16" s="32"/>
@@ -9142,38 +9123,38 @@
       <c r="S16" s="32"/>
     </row>
     <row r="18" spans="14:43" x14ac:dyDescent="0.25">
-      <c r="O18" s="69" t="s">
+      <c r="O18" s="70" t="s">
         <v>131</v>
       </c>
-      <c r="P18" s="69"/>
-      <c r="Q18" s="69"/>
-      <c r="R18" s="69"/>
-      <c r="S18" s="69"/>
-      <c r="T18" s="69"/>
-      <c r="U18" s="69"/>
-      <c r="W18" s="69" t="s">
+      <c r="P18" s="70"/>
+      <c r="Q18" s="70"/>
+      <c r="R18" s="70"/>
+      <c r="S18" s="70"/>
+      <c r="T18" s="70"/>
+      <c r="U18" s="70"/>
+      <c r="W18" s="70" t="s">
         <v>181</v>
       </c>
-      <c r="X18" s="69"/>
-      <c r="Y18" s="69"/>
-      <c r="Z18" s="69"/>
-      <c r="AA18" s="69"/>
-      <c r="AB18" s="69"/>
-      <c r="AC18" s="69"/>
-      <c r="AD18" s="69"/>
-      <c r="AE18" s="69"/>
-      <c r="AF18" s="69"/>
-      <c r="AG18" s="69"/>
-      <c r="AH18" s="69"/>
-      <c r="AI18" s="69"/>
-      <c r="AJ18" s="69"/>
-      <c r="AK18" s="69"/>
-      <c r="AL18" s="69"/>
-      <c r="AM18" s="69"/>
-      <c r="AN18" s="69"/>
-      <c r="AO18" s="69"/>
-      <c r="AP18" s="69"/>
-      <c r="AQ18" s="69"/>
+      <c r="X18" s="70"/>
+      <c r="Y18" s="70"/>
+      <c r="Z18" s="70"/>
+      <c r="AA18" s="70"/>
+      <c r="AB18" s="70"/>
+      <c r="AC18" s="70"/>
+      <c r="AD18" s="70"/>
+      <c r="AE18" s="70"/>
+      <c r="AF18" s="70"/>
+      <c r="AG18" s="70"/>
+      <c r="AH18" s="70"/>
+      <c r="AI18" s="70"/>
+      <c r="AJ18" s="70"/>
+      <c r="AK18" s="70"/>
+      <c r="AL18" s="70"/>
+      <c r="AM18" s="70"/>
+      <c r="AN18" s="70"/>
+      <c r="AO18" s="70"/>
+      <c r="AP18" s="70"/>
+      <c r="AQ18" s="70"/>
     </row>
     <row r="19" spans="14:43" x14ac:dyDescent="0.25">
       <c r="O19" s="46" t="s">
@@ -9334,12 +9315,12 @@
       <c r="S22" s="60" t="s">
         <v>164</v>
       </c>
-      <c r="W22" s="73" t="s">
+      <c r="W22" s="69" t="s">
         <v>203</v>
       </c>
-      <c r="X22" s="73"/>
-      <c r="Y22" s="73"/>
-      <c r="Z22" s="73"/>
+      <c r="X22" s="69"/>
+      <c r="Y22" s="69"/>
+      <c r="Z22" s="69"/>
       <c r="AA22" s="32"/>
       <c r="AB22" s="32"/>
       <c r="AC22" s="32"/>
@@ -9979,16 +9960,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B2:AQ2"/>
+    <mergeCell ref="W18:AQ18"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="W15:Y15"/>
     <mergeCell ref="W22:Z22"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="N3:S3"/>
     <mergeCell ref="O18:U18"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B2:AQ2"/>
-    <mergeCell ref="W18:AQ18"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="W15:Y15"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="K6:L13">
@@ -10017,33 +9998,33 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B7" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B8" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -10076,7 +10057,7 @@
         <v>106</v>
       </c>
       <c r="E3" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -10084,10 +10065,10 @@
         <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E4" s="42" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -10107,7 +10088,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G8" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>212</v>
@@ -10118,13 +10099,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G9" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="I9" s="57" t="s">
         <v>213</v>
       </c>
       <c r="J9" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -10132,7 +10113,7 @@
         <v>209</v>
       </c>
       <c r="J10" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -10140,7 +10121,7 @@
         <v>214</v>
       </c>
       <c r="J11" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -10148,7 +10129,7 @@
         <v>215</v>
       </c>
       <c r="J12" s="42" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -10156,10 +10137,10 @@
         <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E13" s="42" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -10250,7 +10231,7 @@
         <v>207</v>
       </c>
       <c r="K25" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
@@ -10376,7 +10357,7 @@
         <v>78</v>
       </c>
       <c r="E41" s="42" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.25">
@@ -10389,7 +10370,7 @@
         <v>80</v>
       </c>
       <c r="K43" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44" spans="2:11" x14ac:dyDescent="0.25">
@@ -10420,10 +10401,10 @@
         <v>95</v>
       </c>
       <c r="C48" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="G48" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
@@ -10434,7 +10415,7 @@
         <v>220</v>
       </c>
       <c r="G49" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.25">
@@ -10442,7 +10423,7 @@
         <v>97</v>
       </c>
       <c r="G50" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
@@ -10450,13 +10431,13 @@
         <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="D51" t="s">
         <v>221</v>
       </c>
       <c r="G51" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.25">
@@ -10520,7 +10501,7 @@
         <v>90</v>
       </c>
       <c r="K59" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.25">
@@ -10528,7 +10509,7 @@
         <v>91</v>
       </c>
       <c r="E60" s="42" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
@@ -10536,7 +10517,7 @@
         <v>92</v>
       </c>
       <c r="E61" s="42" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
@@ -10552,7 +10533,7 @@
         <v>100</v>
       </c>
       <c r="E63" s="42" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
@@ -10560,7 +10541,7 @@
         <v>101</v>
       </c>
       <c r="E64" s="42" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
@@ -10568,7 +10549,7 @@
         <v>102</v>
       </c>
       <c r="E65" s="42" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
@@ -10588,48 +10569,4 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DC00DF4-147D-4096-AA5C-2C8738D449D0}">
-  <dimension ref="B3:G4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>227</v>
-      </c>
-      <c r="C3" t="s">
-        <v>226</v>
-      </c>
-      <c r="D3" s="42" t="s">
-        <v>228</v>
-      </c>
-      <c r="E3" t="s">
-        <v>229</v>
-      </c>
-      <c r="F3" t="s">
-        <v>230</v>
-      </c>
-      <c r="G3" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>